<commit_message>
Treat ECI transfer as C&V spend, not budget
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XnECCStxZTRunjSaWV1VGN
</commit_message>
<xml_diff>
--- a/budget/CV_Phase_Interactive_Analysis.xlsx
+++ b/budget/CV_Phase_Interactive_Analysis.xlsx
@@ -20,33 +20,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
   <si>
     <t xml:space="preserve">C&amp;V PHASE – INTERACTIVE COST ANALYSIS</t>
   </si>
   <si>
-    <t xml:space="preserve">1. BUDGET (incl. ECI transfer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current C&amp;V budget</t>
+    <t xml:space="preserve">1. BUDGET &amp; SPEND (incl. ECI spend transfer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C&amp;V budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">From budget dashboard (unchanged)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C&amp;V spend to date (dashboard)</t>
   </si>
   <si>
     <t xml:space="preserve">From budget dashboard</t>
   </si>
   <si>
-    <t xml:space="preserve">Transfer from ECI Phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planned transfer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revised C&amp;V budget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spent to date (burn)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Burn % of revised budget</t>
+    <t xml:space="preserve">Spend transferred in from ECI Phase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C&amp;V work logged against ECI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revised C&amp;V spend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Burn % of budget</t>
   </si>
   <si>
     <t xml:space="preserve">Was 54.3% before transfer</t>
@@ -657,7 +660,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>10000</v>
+        <v>44283</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>5</v>
@@ -667,41 +670,41 @@
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="n">
-        <f aca="false">B4+B5</f>
-        <v>91600</v>
+      <c r="B6" s="5" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>44283</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>3</v>
+        <v>8</v>
+      </c>
+      <c r="B7" s="7" t="n">
+        <f aca="false">B5+B6</f>
+        <v>54283</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" s="8" t="n">
-        <f aca="false">B7/B6</f>
-        <v>0.483438864628821</v>
+        <f aca="false">B7/B4</f>
+        <v>0.665232843137255</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B9" s="10" t="n">
-        <f aca="false">B6-B7</f>
-        <v>47317</v>
+        <f aca="false">B4-B7</f>
+        <v>27317</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -709,47 +712,47 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>263</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>526</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B14" s="11" t="n">
         <v>0.8</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">1-B14</f>
@@ -758,7 +761,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B16" s="10" t="n">
         <f aca="false">B12*B14+B13*B15</f>
@@ -770,14 +773,14 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>4</v>
@@ -785,7 +788,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B20" s="13" t="n">
         <v>7</v>
@@ -793,7 +796,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B21" s="14" t="n">
         <f aca="false">B19*B20</f>
@@ -802,28 +805,28 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">B21*B16</f>
         <v>8836.8</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">B7-B22</f>
-        <v>35446.2</v>
+        <v>45446.2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B24" s="12" t="n">
         <v>7</v>
@@ -831,20 +834,20 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B25" s="10" t="n">
         <f aca="false">B23/B24</f>
-        <v>5063.74285714286</v>
+        <v>6492.31428571429</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B26" s="15" t="n">
         <f aca="false">B25/B16</f>
-        <v>16.0448126018468</v>
+        <v>20.5713380409198</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -852,14 +855,14 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B29" s="13" t="n">
         <v>4</v>
@@ -867,7 +870,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B30" s="13" t="n">
         <v>1.5</v>
@@ -875,7 +878,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B31" s="14" t="n">
         <f aca="false">B29+B30</f>
@@ -884,57 +887,57 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B32" s="14" t="n">
         <f aca="false">B26-B31</f>
-        <v>10.5448126018468</v>
+        <v>15.0713380409198</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B33" s="10" t="n">
         <f aca="false">B32*B16</f>
-        <v>3327.94285714286</v>
+        <v>4756.51428571429</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B34" s="16" t="n">
         <f aca="false">B9/B33</f>
-        <v>14.218092687031</v>
+        <v>5.74307115654921</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B35" s="17" t="n">
         <f aca="false">ROUNDDOWN(B34,0)</f>
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B36" s="7" t="n">
         <f aca="false">B9-B35*B33</f>
-        <v>725.80000000001</v>
+        <v>3534.42857142857</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update C&V analysis: latest figures, named rates, 10-15 hr scenario range
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XnECCStxZTRunjSaWV1VGN
</commit_message>
<xml_diff>
--- a/budget/CV_Phase_Interactive_Analysis.xlsx
+++ b/budget/CV_Phase_Interactive_Analysis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
   <si>
     <t xml:space="preserve">C&amp;V PHASE – INTERACTIVE COST ANALYSIS</t>
   </si>
@@ -37,7 +37,7 @@
     <t xml:space="preserve">C&amp;V spend to date (dashboard)</t>
   </si>
   <si>
-    <t xml:space="preserve">From budget dashboard</t>
+    <t xml:space="preserve">From latest budget dashboard</t>
   </si>
   <si>
     <t xml:space="preserve">Spend transferred in from ECI Phase</t>
@@ -52,31 +52,28 @@
     <t xml:space="preserve">Burn % of budget</t>
   </si>
   <si>
-    <t xml:space="preserve">Was 54.3% before transfer</t>
-  </si>
-  <si>
     <t xml:space="preserve">Remaining budget</t>
   </si>
   <si>
     <t xml:space="preserve">2. RATES</t>
   </si>
   <si>
-    <t xml:space="preserve">Your hourly rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provided by you</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Boss's hourly rate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Your share of time</t>
+    <t xml:space="preserve">Alycia hourly rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provided by Alycia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeffrey hourly rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alycia share of time</t>
   </si>
   <si>
     <t xml:space="preserve">Planning split</t>
   </si>
   <si>
-    <t xml:space="preserve">Boss's share of time</t>
+    <t xml:space="preserve">Jeffrey share of time</t>
   </si>
   <si>
     <t xml:space="preserve">Blended hourly rate</t>
@@ -112,7 +109,7 @@
     <t xml:space="preserve">Average hours per interactive</t>
   </si>
   <si>
-    <t xml:space="preserve">4. FUTURE INTERACTIVES (reduced rate)</t>
+    <t xml:space="preserve">4. FUTURE ESTIMATE – HISTORIC BASIS (upper end)</t>
   </si>
   <si>
     <t xml:space="preserve">Hours saved – no longer attending interactive</t>
@@ -121,28 +118,49 @@
     <t xml:space="preserve">Hours saved – no early admin/challenges</t>
   </si>
   <si>
-    <t xml:space="preserve">Total hours removed per interactive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Future hours per interactive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Future cost per interactive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Future interactives remaining budget covers (exact)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Future interactives we can support (whole)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budget left over after those interactives</t>
+    <t xml:space="preserve">Future hours per interactive (historic avg less savings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most recent interactive – actual hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest interactive took ~10 hrs (lower end)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. HOW MANY MORE INTERACTIVES? (range)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best case (recent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Midpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conservative (historic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hours per interactive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost per interactive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interactives remaining budget covers (exact)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Interactives we can support (whole)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget left over</t>
   </si>
   <si>
     <t xml:space="preserve">Legend: yellow cells with blue text are inputs – change them and everything recalculates. Shaded blue rows are key results.</t>
   </si>
   <si>
     <t xml:space="preserve">Assumption: past hours are estimated by dividing past spend by the 80/20 blended rate, as the actual historic staff mix isn't known.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best case uses the most recent interactive (~10 hrs); conservative uses the historic average less the 5.5 hrs of savings.</t>
   </si>
 </sst>
 </file>
@@ -155,7 +173,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.00&quot; hrs&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0&quot; hrs&quot;"/>
     <numFmt numFmtId="170" formatCode="0.00"/>
   </numFmts>
   <fonts count="11">
@@ -292,7 +310,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -354,6 +372,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -621,12 +643,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -643,6 +665,8 @@
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
@@ -651,7 +675,7 @@
       <c r="B4" s="5" t="n">
         <v>81600</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>3</v>
       </c>
     </row>
@@ -660,9 +684,9 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>44283</v>
-      </c>
-      <c r="C5" s="6" t="s">
+        <v>44809</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -673,7 +697,7 @@
       <c r="B6" s="5" t="n">
         <v>10000</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -683,7 +707,7 @@
       </c>
       <c r="B7" s="7" t="n">
         <f aca="false">B5+B6</f>
-        <v>54283</v>
+        <v>54809</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -692,19 +716,16 @@
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">B7/B4</f>
-        <v>0.665232843137255</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>10</v>
+        <v>0.671678921568627</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">B4-B7</f>
-        <v>27317</v>
+        <v>26791</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -712,47 +733,49 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>263</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>14</v>
+      <c r="E12" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B13" s="5" t="n">
         <v>526</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>14</v>
+      <c r="E13" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="11" t="n">
         <v>0.8</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>17</v>
+      <c r="E14" s="6" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">1-B14</f>
@@ -761,7 +784,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" s="10" t="n">
         <f aca="false">B12*B14+B13*B15</f>
@@ -773,14 +796,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>4</v>
@@ -788,7 +813,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B20" s="13" t="n">
         <v>7</v>
@@ -796,7 +821,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B21" s="14" t="n">
         <f aca="false">B19*B20</f>
@@ -805,28 +830,28 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">B21*B16</f>
         <v>8836.8</v>
       </c>
-      <c r="C22" s="6" t="s">
-        <v>25</v>
+      <c r="E22" s="6" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" s="7" t="n">
         <f aca="false">B7-B22</f>
-        <v>45446.2</v>
+        <v>45972.2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B24" s="12" t="n">
         <v>7</v>
@@ -834,20 +859,20 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B25" s="10" t="n">
         <f aca="false">B23/B24</f>
-        <v>6492.31428571429</v>
+        <v>6567.45714285714</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B26" s="15" t="n">
         <f aca="false">B25/B16</f>
-        <v>20.5713380409198</v>
+        <v>20.809433279015</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -855,14 +880,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B29" s="13" t="n">
         <v>4</v>
@@ -870,74 +897,151 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="13" t="n">
         <v>1.5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31" s="14" t="n">
-        <f aca="false">B29+B30</f>
-        <v>5.5</v>
+      <c r="A31" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B31" s="15" t="n">
+        <f aca="false">B26-B29-B30</f>
+        <v>15.309433279015</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="14" t="n">
-        <f aca="false">B26-B31</f>
-        <v>15.0713380409198</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="9" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="10" t="n">
-        <f aca="false">B32*B16</f>
-        <v>4756.51428571429</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="16"/>
+      <c r="B35" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="B34" s="16" t="n">
-        <f aca="false">B9/B33</f>
-        <v>5.74307115654921</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9" t="s">
+      <c r="C35" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B35" s="17" t="n">
-        <f aca="false">ROUNDDOWN(B34,0)</f>
-        <v>5</v>
+      <c r="D35" s="16" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36" s="7" t="n">
-        <f aca="false">B9-B35*B33</f>
-        <v>3534.42857142857</v>
+        <v>39</v>
+      </c>
+      <c r="B36" s="14" t="n">
+        <f aca="false">B32</f>
+        <v>10</v>
+      </c>
+      <c r="C36" s="14" t="n">
+        <f aca="false">AVERAGE(B36,D36)</f>
+        <v>12.6547166395075</v>
+      </c>
+      <c r="D36" s="14" t="n">
+        <f aca="false">B31</f>
+        <v>15.309433279015</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <f aca="false">B36*$B$16</f>
+        <v>3156</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <f aca="false">C36*$B$16</f>
+        <v>3993.82857142857</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <f aca="false">D36*$B$16</f>
+        <v>4831.65714285714</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="18" t="s">
-        <v>39</v>
+      <c r="A38" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B38" s="17" t="n">
+        <f aca="false">$B$9/B37</f>
+        <v>8.48891001267427</v>
+      </c>
+      <c r="C38" s="17" t="n">
+        <f aca="false">$B$9/C37</f>
+        <v>6.70809963944371</v>
+      </c>
+      <c r="D38" s="17" t="n">
+        <f aca="false">$B$9/D37</f>
+        <v>5.54488847363815</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="18" t="s">
-        <v>40</v>
+      <c r="A39" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="18" t="n">
+        <f aca="false">ROUNDDOWN(B38,0)</f>
+        <v>8</v>
+      </c>
+      <c r="C39" s="18" t="n">
+        <f aca="false">ROUNDDOWN(C38,0)</f>
+        <v>6</v>
+      </c>
+      <c r="D39" s="18" t="n">
+        <f aca="false">ROUNDDOWN(D38,0)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <f aca="false">$B$9-B39*B37</f>
+        <v>1543</v>
+      </c>
+      <c r="C40" s="7" t="n">
+        <f aca="false">$B$9-C39*C37</f>
+        <v>2828.02857142857</v>
+      </c>
+      <c r="D40" s="7" t="n">
+        <f aca="false">$B$9-D39*D37</f>
+        <v>2632.71428571429</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="19" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="19" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Increase future per-interactive savings to 6.5 hrs (no debrief doc)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XnECCStxZTRunjSaWV1VGN
</commit_message>
<xml_diff>
--- a/budget/CV_Phase_Interactive_Analysis.xlsx
+++ b/budget/CV_Phase_Interactive_Analysis.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t xml:space="preserve">C&amp;V PHASE – INTERACTIVE COST ANALYSIS</t>
   </si>
@@ -118,7 +118,10 @@
     <t xml:space="preserve">Hours saved – no early admin/challenges</t>
   </si>
   <si>
-    <t xml:space="preserve">Future hours per interactive (historic avg less savings)</t>
+    <t xml:space="preserve">Hours saved – no debrief document/guidance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Future hours per interactive (historic avg less 6.5 hrs savings)</t>
   </si>
   <si>
     <t xml:space="preserve">Most recent interactive – actual hours</t>
@@ -160,7 +163,7 @@
     <t xml:space="preserve">Assumption: past hours are estimated by dividing past spend by the 80/20 blended rate, as the actual historic staff mix isn't known.</t>
   </si>
   <si>
-    <t xml:space="preserve">Best case uses the most recent interactive (~10 hrs); conservative uses the historic average less the 5.5 hrs of savings.</t>
+    <t xml:space="preserve">Best case uses the most recent interactive (~10 hrs); conservative uses the historic average less the 6.5 hrs of savings.</t>
   </si>
 </sst>
 </file>
@@ -643,7 +646,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="54"/>
@@ -904,134 +907,137 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="15" t="n">
-        <f aca="false">B26-B29-B30</f>
-        <v>15.309433279015</v>
+      <c r="B31" s="13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B32" s="13" t="n">
+      <c r="B32" s="15" t="n">
+        <f aca="false">B26-B29-B30-B31</f>
+        <v>14.309433279015</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B33" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="E32" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
+      <c r="E33" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4"/>
-      <c r="E34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="16"/>
-      <c r="B35" s="16" t="s">
+      <c r="A35" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="C35" s="16" t="s">
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="16"/>
+      <c r="B36" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="D35" s="16" t="s">
+      <c r="C36" s="16" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="D36" s="16" t="s">
         <v>39</v>
-      </c>
-      <c r="B36" s="14" t="n">
-        <f aca="false">B32</f>
-        <v>10</v>
-      </c>
-      <c r="C36" s="14" t="n">
-        <f aca="false">AVERAGE(B36,D36)</f>
-        <v>12.6547166395075</v>
-      </c>
-      <c r="D36" s="14" t="n">
-        <f aca="false">B31</f>
-        <v>15.309433279015</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B37" s="7" t="n">
-        <f aca="false">B36*$B$16</f>
-        <v>3156</v>
-      </c>
-      <c r="C37" s="7" t="n">
-        <f aca="false">C36*$B$16</f>
-        <v>3993.82857142857</v>
-      </c>
-      <c r="D37" s="7" t="n">
-        <f aca="false">D36*$B$16</f>
-        <v>4831.65714285714</v>
+      <c r="B37" s="14" t="n">
+        <f aca="false">B33</f>
+        <v>10</v>
+      </c>
+      <c r="C37" s="14" t="n">
+        <f aca="false">AVERAGE(B37,D37)</f>
+        <v>12.1547166395075</v>
+      </c>
+      <c r="D37" s="14" t="n">
+        <f aca="false">B32</f>
+        <v>14.309433279015</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="17" t="n">
-        <f aca="false">$B$9/B37</f>
+      <c r="B38" s="7" t="n">
+        <f aca="false">B37*$B$16</f>
+        <v>3156</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <f aca="false">C37*$B$16</f>
+        <v>3836.02857142857</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <f aca="false">D37*$B$16</f>
+        <v>4516.05714285714</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B39" s="17" t="n">
+        <f aca="false">$B$9/B38</f>
         <v>8.48891001267427</v>
       </c>
-      <c r="C38" s="17" t="n">
-        <f aca="false">$B$9/C37</f>
-        <v>6.70809963944371</v>
-      </c>
-      <c r="D38" s="17" t="n">
-        <f aca="false">$B$9/D37</f>
-        <v>5.54488847363815</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="18" t="n">
-        <f aca="false">ROUNDDOWN(B38,0)</f>
+      <c r="C39" s="17" t="n">
+        <f aca="false">$B$9/C38</f>
+        <v>6.98404599995531</v>
+      </c>
+      <c r="D39" s="17" t="n">
+        <f aca="false">$B$9/D38</f>
+        <v>5.932387291063</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="18" t="n">
+        <f aca="false">ROUNDDOWN(B39,0)</f>
         <v>8</v>
       </c>
-      <c r="C39" s="18" t="n">
-        <f aca="false">ROUNDDOWN(C38,0)</f>
+      <c r="C40" s="18" t="n">
+        <f aca="false">ROUNDDOWN(C39,0)</f>
         <v>6</v>
       </c>
-      <c r="D39" s="18" t="n">
-        <f aca="false">ROUNDDOWN(D38,0)</f>
+      <c r="D40" s="18" t="n">
+        <f aca="false">ROUNDDOWN(D39,0)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <f aca="false">$B$9-B39*B37</f>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B41" s="7" t="n">
+        <f aca="false">$B$9-B40*B38</f>
         <v>1543</v>
       </c>
-      <c r="C40" s="7" t="n">
-        <f aca="false">$B$9-C39*C37</f>
-        <v>2828.02857142857</v>
-      </c>
-      <c r="D40" s="7" t="n">
-        <f aca="false">$B$9-D39*D37</f>
-        <v>2632.71428571429</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="19" t="s">
-        <v>44</v>
+      <c r="C41" s="7" t="n">
+        <f aca="false">$B$9-C40*C38</f>
+        <v>3774.82857142857</v>
+      </c>
+      <c r="D41" s="7" t="n">
+        <f aca="false">$B$9-D40*D38</f>
+        <v>4210.71428571429</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1042,6 +1048,11 @@
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
         <v>46</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="19" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Round future interactive counts to nearest whole number
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XnECCStxZTRunjSaWV1VGN
</commit_message>
<xml_diff>
--- a/budget/CV_Phase_Interactive_Analysis.xlsx
+++ b/budget/CV_Phase_Interactive_Analysis.xlsx
@@ -151,10 +151,10 @@
     <t xml:space="preserve">Interactives remaining budget covers (exact)</t>
   </si>
   <si>
-    <t xml:space="preserve">Interactives we can support (whole)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budget left over</t>
+    <t xml:space="preserve">Interactives we can support (rounded to nearest)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget left over / (overrun)</t>
   </si>
   <si>
     <t xml:space="preserve">Legend: yellow cells with blue text are inputs – change them and everything recalculates. Shaded blue rows are key results.</t>
@@ -163,7 +163,7 @@
     <t xml:space="preserve">Assumption: past hours are estimated by dividing past spend by the 80/20 blended rate, as the actual historic staff mix isn't known.</t>
   </si>
   <si>
-    <t xml:space="preserve">Best case uses the most recent interactive (~10 hrs); conservative uses the historic average less the 6.5 hrs of savings.</t>
+    <t xml:space="preserve">Best case uses the most recent interactive (~10 hrs); conservative uses the historic average less the 6.5 hrs of savings. Counts are rounded to the nearest whole interactive, so a small overrun (in brackets) may show.</t>
   </si>
 </sst>
 </file>
@@ -1011,16 +1011,16 @@
         <v>43</v>
       </c>
       <c r="B40" s="18" t="n">
-        <f aca="false">ROUNDDOWN(B39,0)</f>
+        <f aca="false">ROUND(B39,0)</f>
         <v>8</v>
       </c>
       <c r="C40" s="18" t="n">
-        <f aca="false">ROUNDDOWN(C39,0)</f>
+        <f aca="false">ROUND(C39,0)</f>
+        <v>7</v>
+      </c>
+      <c r="D40" s="18" t="n">
+        <f aca="false">ROUND(D39,0)</f>
         <v>6</v>
-      </c>
-      <c r="D40" s="18" t="n">
-        <f aca="false">ROUNDDOWN(D39,0)</f>
-        <v>5</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1033,11 +1033,11 @@
       </c>
       <c r="C41" s="7" t="n">
         <f aca="false">$B$9-C40*C38</f>
-        <v>3774.82857142857</v>
+        <v>-61.1999999999971</v>
       </c>
       <c r="D41" s="7" t="n">
         <f aca="false">$B$9-D40*D38</f>
-        <v>4210.71428571429</v>
+        <v>-305.342857142852</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>